<commit_message>
feat: implemented proper teamlead and reporting manager
</commit_message>
<xml_diff>
--- a/EmployeeSummary_transformed.xlsx
+++ b/EmployeeSummary_transformed.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH384"/>
+  <dimension ref="A1:AI384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,6 +591,11 @@
           <t>PermanentAddress</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Manager_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -731,6 +736,7 @@
           <t>House# 832, Road # 5, Baitul Aman Housing, Adabar, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -867,6 +873,7 @@
           <t>Krishi Market, Mohammadpur, Dhaka -1207</t>
         </is>
       </c>
+      <c r="AI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1003,6 +1010,7 @@
           <t>34/22, Pallabi, Mirpur-12, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1143,6 +1151,7 @@
           <t>D-2, Cha-151/152, Mohakhali, Dhaka-1213</t>
         </is>
       </c>
+      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1279,6 +1288,7 @@
           <t>KA-49,Afsar Villa,3rd Floor,Moddhopara,Khilkhet,Dhaka-1229</t>
         </is>
       </c>
+      <c r="AI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1419,6 +1429,7 @@
           <t>Flat # 501, H # 10, Level - 5, Block # H, Pallabi Extension R/A, Section-12, Mirpur Dhaka - 1216.</t>
         </is>
       </c>
+      <c r="AI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1553,6 +1564,9 @@
           <t>34,35,35/1, 'Ideal Panorama', Shantinagar, Dhaka-1217</t>
         </is>
       </c>
+      <c r="AI8" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1687,6 +1701,9 @@
           <t>1/8, Tolarbag, Mirpur-1, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI9" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1813,6 +1830,9 @@
           <t xml:space="preserve">Moyuri Aparetment, 90/1 Boro Moghbazar, Ramnha, Dhaka - 1217. </t>
         </is>
       </c>
+      <c r="AI10" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1963,6 +1983,9 @@
           <t>157/A, West Rampura, Dhaka</t>
         </is>
       </c>
+      <c r="AI11" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2115,6 +2138,9 @@
           <t xml:space="preserve">House-120 (3rd Floor), Flat-3A, Mollartek Udayan High School &amp; College Road, Dokhenkhan, Uttara, Dhaka </t>
         </is>
       </c>
+      <c r="AI12" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2261,6 +2287,9 @@
           <t>Village- Jatpur, PO- Jatpur Bazar, PS- Tala, Satkhira</t>
         </is>
       </c>
+      <c r="AI13" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2410,6 +2439,9 @@
         <is>
           <t>House-152 (6th Floor), West Nakhalpara, Tejgaon, Dhaka</t>
         </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -2497,6 +2529,7 @@
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2615,6 +2648,7 @@
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2729,6 +2763,7 @@
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2817,6 +2852,7 @@
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2953,6 +2989,9 @@
           <t>House No. 402, 404 (Flat B-2), Road No. 06, Mirpur DOHS, Mirpur-12, Dhaka</t>
         </is>
       </c>
+      <c r="AI19" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3074,6 +3113,9 @@
         <is>
           <t>House # 45, Road # 7, Banani, Dhaka</t>
         </is>
+      </c>
+      <c r="AI20" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="21">
@@ -3201,6 +3243,9 @@
           <t>House - 09, Road -12, Sector - 03, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI21" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3337,6 +3382,7 @@
           <t>House No. 18, Road No. 9-D, Sector no. 5, Uttara, Dhaka-1230</t>
         </is>
       </c>
+      <c r="AI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3465,6 +3511,7 @@
           <t>H-27, Road No 22, Malibag Choudhury Para, Khilgaon, KhilgaonTSO, Khilgaon</t>
         </is>
       </c>
+      <c r="AI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3595,6 +3642,7 @@
           <t>Rankin street, wari, Dhaka-1203</t>
         </is>
       </c>
+      <c r="AI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3729,6 +3777,9 @@
           <t>House#4, Road#21, Gulshan - 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI25" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3863,6 +3914,9 @@
           <t>111/4, 3rd Floor, PatwaryGoli, East Basaboo, Sabujbagh, Dhaka.</t>
         </is>
       </c>
+      <c r="AI26" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3999,6 +4053,7 @@
           <t>JMI Osman Gani Villa, Flat# 8B,Green Corner, Green Road, Kolabagan, Dhaka1205</t>
         </is>
       </c>
+      <c r="AI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -4139,6 +4194,7 @@
           <t>Bondhu Nibash, House#01, Road# 04, Block # A, Nobodoy Housing, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4275,6 +4331,9 @@
           <t>169/8/B West Dolaipar, (5th Floor), Panthonibash, Shampur, Dhaka-1204</t>
         </is>
       </c>
+      <c r="AI29" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4411,6 +4470,7 @@
           <t>272/3, malibagh, Dhaka</t>
         </is>
       </c>
+      <c r="AI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4545,6 +4605,9 @@
           <t>Road # 08, House # 15, Merul Badda DIT Project, Dhaka</t>
         </is>
       </c>
+      <c r="AI31" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4675,6 +4738,9 @@
           <t>House#4, Road#21, Gulshan - 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI32" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4805,6 +4871,9 @@
           <t>Road#11, House#11, Baridhara, Dhaka</t>
         </is>
       </c>
+      <c r="AI33" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4935,6 +5004,9 @@
           <t>House#6, 12th floor, lane 13, Block A, Mirpur</t>
         </is>
       </c>
+      <c r="AI34" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -5071,6 +5143,7 @@
           <t>House#13, Road#12, Dhanmondi, Dhaka</t>
         </is>
       </c>
+      <c r="AI35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -5207,6 +5280,7 @@
           <t>House#13, Road#12, Dhanmondi, Dhaka</t>
         </is>
       </c>
+      <c r="AI36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5343,6 +5417,7 @@
           <t>House#13, Road#12, Dhanmondi, Dhaka</t>
         </is>
       </c>
+      <c r="AI37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -5475,6 +5550,7 @@
           <t>618/A, Middle Monipur, Mirpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -5615,6 +5691,7 @@
           <t>Road # 18, House # 30, Sector 7, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -5755,6 +5832,7 @@
           <t>House#4, Road#21, Gulshan - 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -5887,6 +5965,7 @@
           <t>House#58/1, Lichu Bagan, Mir Akhter Store, Shawra, Lichubagan, Dhaka</t>
         </is>
       </c>
+      <c r="AI41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -6023,6 +6102,7 @@
           <t>M-36, GF, Noorjahan Road, Mohammadpur, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -6155,6 +6235,7 @@
           <t>Road#11, House#11, Baridhara, Dhaka</t>
         </is>
       </c>
+      <c r="AI43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -6287,6 +6368,7 @@
           <t>H-1084/1085, R-21, Khilgaon, Tilpara, Dhaka-1230</t>
         </is>
       </c>
+      <c r="AI44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -6413,6 +6495,7 @@
           <t>MD's House</t>
         </is>
       </c>
+      <c r="AI45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -6495,6 +6578,7 @@
       <c r="AF46" t="inlineStr"/>
       <c r="AG46" t="inlineStr"/>
       <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -6625,6 +6709,9 @@
           <t>House#5, Road#21, Gulshan 1- Dhaka</t>
         </is>
       </c>
+      <c r="AI47" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -6759,6 +6846,9 @@
           <t>House # 17/4, New Baily Road, Dhaka</t>
         </is>
       </c>
+      <c r="AI48" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -6893,6 +6983,9 @@
           <t>Mita Manzil, 250/A, South Jatrabari, 1st Floor, Dhaka-1204</t>
         </is>
       </c>
+      <c r="AI49" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -7025,6 +7118,7 @@
           <t>House#34A, Gulbbagh, Dhaka</t>
         </is>
       </c>
+      <c r="AI50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -7157,6 +7251,7 @@
           <t>180 Bosila, Mohammadpur</t>
         </is>
       </c>
+      <c r="AI51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -7291,6 +7386,9 @@
           <t>House 1058, Road 7, Avenue 8, Mirpur DOHS, Mirpur 12, Dhaka 1216</t>
         </is>
       </c>
+      <c r="AI52" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -7421,6 +7519,9 @@
           <t>House# 72, Sardar Villa, Taltola, Agargaon, Dhaka</t>
         </is>
       </c>
+      <c r="AI53" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -7557,6 +7658,7 @@
           <t>House#27, Middle Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -7687,6 +7789,9 @@
           <t>Satmasjid Road, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI55" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -7817,6 +7922,9 @@
           <t>House#4, road#21, Gulshan - 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI56" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -7949,6 +8057,7 @@
           <t>MD's House</t>
         </is>
       </c>
+      <c r="AI57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8085,6 +8194,7 @@
           <t>363 Uttar Mugrakul, Jatramura, Tarabo Pourasava, Rupgonj, Narayangonj</t>
         </is>
       </c>
+      <c r="AI58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -8217,6 +8327,7 @@
           <t>Modhubagh 1 No. Lane, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -8351,6 +8462,9 @@
           <t>House#57/A Maniknagar, Mugda, jatrabari, Dhaka</t>
         </is>
       </c>
+      <c r="AI60" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -8487,6 +8601,7 @@
           <t>House#3/14, Block # A, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -8623,6 +8738,7 @@
           <t>Addeen Hospital, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -8709,6 +8825,9 @@
       <c r="AF63" t="inlineStr"/>
       <c r="AG63" t="inlineStr"/>
       <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -8859,6 +8978,9 @@
           <t>Ka 26, Nadda Sharkarbari, Gulshan-2, Dhaka</t>
         </is>
       </c>
+      <c r="AI64" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -9010,6 +9132,9 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI65" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -9161,6 +9286,7 @@
           <t>Flat-B2, House-402, Road-6, Avenue-3, Mirpur DOHS, Pallabi, Dhaka</t>
         </is>
       </c>
+      <c r="AI66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -9293,6 +9419,7 @@
           <t>House-059, Jomader Bari Road, Western Para, PS-Lalmohon, Bhola</t>
         </is>
       </c>
+      <c r="AI67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9439,6 +9566,9 @@
           <t>Village-Shampur, PO-Charmastul, Doulatpur, Manikganj</t>
         </is>
       </c>
+      <c r="AI68" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9579,6 +9709,7 @@
           <t>49/50 Hossaini Dalan, Dhaka</t>
         </is>
       </c>
+      <c r="AI69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -9713,6 +9844,9 @@
           <t>House - C, Road - 24, Madina Nagar, Avenue: 5, Mirpur -11, Dhaka- 1216</t>
         </is>
       </c>
+      <c r="AI70" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -9849,6 +9983,7 @@
           <t>H-97-1/B,Chairman Goli,Shankar, Dhanmondi,Dhaka</t>
         </is>
       </c>
+      <c r="AI71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -9983,6 +10118,9 @@
           <t>House: 291, Flat: 4A, Tali Office Road, Rayer Bazar, Dhaka-1209</t>
         </is>
       </c>
+      <c r="AI72" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10123,6 +10261,7 @@
           <t>F-A3,H-17,R-02,Turag City, Shahali Thana, Mirpur-01, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10255,6 +10394,7 @@
           <t>Moghbazar, Malibagh, Dhaka</t>
         </is>
       </c>
+      <c r="AI74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10367,6 +10507,7 @@
           <t>Flat- A4, Shelter Heritage, Plot-2, Kallyanpur Main Road, Dhaka</t>
         </is>
       </c>
+      <c r="AI75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10507,6 +10648,7 @@
           <t xml:space="preserve">7C/47, Hashem Bari,Indira Road,Firmgate Dhaka </t>
         </is>
       </c>
+      <c r="AI76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10647,6 +10789,7 @@
           <t>H:64 (2nd Floor), R:07, DIT Project, Merul Badda, Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10787,6 +10930,7 @@
           <t>23/2 West Nakhal Para, Tejgaon, Dhaka-1215</t>
         </is>
       </c>
+      <c r="AI78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10927,6 +11071,7 @@
           <t>House#57,Road-3/A,FLat#B-3,Dhanmondi,Dhaka-1209</t>
         </is>
       </c>
+      <c r="AI79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11067,6 +11212,7 @@
           <t>1/G, Paribagh Apartments, Flat #B4, Paribagh, Shahbag, Dhaka</t>
         </is>
       </c>
+      <c r="AI80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -11195,6 +11341,7 @@
           <t xml:space="preserve">Holding  No-1069   Block -B, PO-Merajnagor, PS-Kodomtoli, Dhaka -1362 </t>
         </is>
       </c>
+      <c r="AI81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11335,6 +11482,7 @@
           <t>West Hazinagar, Sarulia, Demra</t>
         </is>
       </c>
+      <c r="AI82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11465,6 +11613,9 @@
           <t>Badda, Gulshan, Dhaka</t>
         </is>
       </c>
+      <c r="AI83" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11611,6 +11762,9 @@
           <t>H-7, R-9, Block-C, Sec-6, Mirpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI84" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11759,6 +11913,9 @@
           <t>18, Shekhertek, Road-05, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI85" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11907,6 +12064,7 @@
           <t>House-444, Mokki Mosque Road, Rampura, Dhaka</t>
         </is>
       </c>
+      <c r="AI86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12053,6 +12211,9 @@
           <t xml:space="preserve">House117, Khan Villa, Ananda Bazar, West Shewrapara, Mirpur, Dhaka </t>
         </is>
       </c>
+      <c r="AI87" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -12199,6 +12360,9 @@
           <t>H-20, R-1, Block-B, Banasree, Dhaka</t>
         </is>
       </c>
+      <c r="AI88" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -12333,6 +12497,9 @@
           <t>Apt. 401, House 3, Road 1, Block B, Niketon, Gulshan, Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI89" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12473,6 +12640,7 @@
           <t>House 413 (Level 6), Road 7, Avenue 3, DOHS, Mirpur, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12591,6 +12759,9 @@
           <t>Anantopur, Mullargaon,Sylhet Sadar, Sylhet.</t>
         </is>
       </c>
+      <c r="AI91" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -12725,6 +12896,9 @@
           <t>149/B Khilgaon Chowdhury para, Dhaka</t>
         </is>
       </c>
+      <c r="AI92" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -12865,6 +13039,7 @@
           <t>House 10, Road 1/C, Block B, Nobodoy Housing Society, Mohammadpur, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -13001,6 +13176,7 @@
           <t>B-store, BTCL Colony, karail, Banani Road-5, Dhaka 1213</t>
         </is>
       </c>
+      <c r="AI94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -13141,6 +13317,7 @@
           <t>House-08, Road-07, Block-Kha, P C Culture Housing, Shekhertek, Adabor, Dhaka.</t>
         </is>
       </c>
+      <c r="AI95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -13281,6 +13458,7 @@
           <t>House No- 271, Block-B, Khilgaon, Taltola, Dhaka</t>
         </is>
       </c>
+      <c r="AI96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -13421,6 +13599,7 @@
           <t>Uttara Model Town, Dhaka</t>
         </is>
       </c>
+      <c r="AI97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -13561,6 +13740,7 @@
           <t>FLAT-4B,HOUSE:2,ROAD:1/A,BLOCK:B,NOBODOY HOUSING,Mohammadpur</t>
         </is>
       </c>
+      <c r="AI98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -13697,6 +13877,7 @@
           <t>Flat B4, House#15, Road#13, Sector#6, Uttara, Dhaka, 1230</t>
         </is>
       </c>
+      <c r="AI99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -13833,6 +14014,7 @@
           <t>House- 69/C/3, Road-6/A Dhanmondi R/A, Dhaka-1209</t>
         </is>
       </c>
+      <c r="AI100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -13986,6 +14168,9 @@
           <t>415/1, Nur-E-Modina Jame Mosjid Road, Kawlar, Dhaka</t>
         </is>
       </c>
+      <c r="AI101" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -14134,6 +14319,7 @@
           <t xml:space="preserve">House-21, Mina Kunjo, Boroitola Bazar, Khilbarir Tek, Vatara, Dhaka </t>
         </is>
       </c>
+      <c r="AI102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -14220,6 +14406,7 @@
       <c r="AF103" t="inlineStr"/>
       <c r="AG103" t="inlineStr"/>
       <c r="AH103" t="inlineStr"/>
+      <c r="AI103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -14316,6 +14503,7 @@
           <t>65, Sir Iqbal Road, Batipara, Khulna.</t>
         </is>
       </c>
+      <c r="AI104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -14400,6 +14588,7 @@
       <c r="AF105" t="inlineStr"/>
       <c r="AG105" t="inlineStr"/>
       <c r="AH105" t="inlineStr"/>
+      <c r="AI105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -14536,6 +14725,7 @@
       </c>
       <c r="AG106" t="inlineStr"/>
       <c r="AH106" t="inlineStr"/>
+      <c r="AI106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -14680,6 +14870,7 @@
           <t>18/B Malibagh, Chowdhuripara, Dhaka</t>
         </is>
       </c>
+      <c r="AI107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -14828,6 +15019,7 @@
           <t>Tongi, Millget</t>
         </is>
       </c>
+      <c r="AI108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -14976,6 +15168,7 @@
           <t>Kalachadpur, Gulshan 2, Dhaka - 1212</t>
         </is>
       </c>
+      <c r="AI109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -15102,6 +15295,7 @@
 Uttar Khan, Dhaka .</t>
         </is>
       </c>
+      <c r="AI110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -15218,6 +15412,7 @@
       <c r="AF111" t="inlineStr"/>
       <c r="AG111" t="inlineStr"/>
       <c r="AH111" t="inlineStr"/>
+      <c r="AI111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -15300,6 +15495,7 @@
       <c r="AF112" t="inlineStr"/>
       <c r="AG112" t="inlineStr"/>
       <c r="AH112" t="inlineStr"/>
+      <c r="AI112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -15382,6 +15578,7 @@
       <c r="AF113" t="inlineStr"/>
       <c r="AG113" t="inlineStr"/>
       <c r="AH113" t="inlineStr"/>
+      <c r="AI113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -15464,6 +15661,7 @@
       <c r="AF114" t="inlineStr"/>
       <c r="AG114" t="inlineStr"/>
       <c r="AH114" t="inlineStr"/>
+      <c r="AI114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -15546,6 +15744,7 @@
       <c r="AF115" t="inlineStr"/>
       <c r="AG115" t="inlineStr"/>
       <c r="AH115" t="inlineStr"/>
+      <c r="AI115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -15628,6 +15827,7 @@
       <c r="AF116" t="inlineStr"/>
       <c r="AG116" t="inlineStr"/>
       <c r="AH116" t="inlineStr"/>
+      <c r="AI116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -15710,6 +15910,7 @@
       <c r="AF117" t="inlineStr"/>
       <c r="AG117" t="inlineStr"/>
       <c r="AH117" t="inlineStr"/>
+      <c r="AI117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -15792,6 +15993,7 @@
       <c r="AF118" t="inlineStr"/>
       <c r="AG118" t="inlineStr"/>
       <c r="AH118" t="inlineStr"/>
+      <c r="AI118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -15874,6 +16076,7 @@
       <c r="AF119" t="inlineStr"/>
       <c r="AG119" t="inlineStr"/>
       <c r="AH119" t="inlineStr"/>
+      <c r="AI119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -15956,6 +16159,7 @@
       <c r="AF120" t="inlineStr"/>
       <c r="AG120" t="inlineStr"/>
       <c r="AH120" t="inlineStr"/>
+      <c r="AI120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -16038,6 +16242,7 @@
       <c r="AF121" t="inlineStr"/>
       <c r="AG121" t="inlineStr"/>
       <c r="AH121" t="inlineStr"/>
+      <c r="AI121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -16174,6 +16379,7 @@
           <t>20/3A west Dolaipar, Dhaka - 1204</t>
         </is>
       </c>
+      <c r="AI122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -16318,6 +16524,7 @@
           <t>Gp kha-13, South Kuril, Dhaka 1212</t>
         </is>
       </c>
+      <c r="AI123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -16469,6 +16676,7 @@
           <t>k-55/1 kalachadpur Gulshan - 2 Dhaka- 1212</t>
         </is>
       </c>
+      <c r="AI124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -16613,6 +16821,7 @@
           <t xml:space="preserve">Board Bazar, Gazipur. </t>
         </is>
       </c>
+      <c r="AI125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -16761,6 +16970,7 @@
           <t>Dogair South-West para, Milon Road, Sharulia, Demra, Dhaka</t>
         </is>
       </c>
+      <c r="AI126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -16909,6 +17119,7 @@
           <t>Kalachadpur, Nodda, Gulshan 2, Dhaka- 1212</t>
         </is>
       </c>
+      <c r="AI127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17057,6 +17268,7 @@
           <t>1218 Sher-e- Bangla Road, Shahi Mosjid Goli, Katasur, Mohammadpur, Dhaka 1207</t>
         </is>
       </c>
+      <c r="AI128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17201,6 +17413,7 @@
           <t>3/3 charakghata, Tali Office, Dhaka 1209, Hazaribag, Dhaka</t>
         </is>
       </c>
+      <c r="AI129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17352,6 +17565,7 @@
           <t>ka-55/B Ashrat Manjil</t>
         </is>
       </c>
+      <c r="AI130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -17500,6 +17714,7 @@
           <t>137/17 2nd colony, mirpur-1, Dhaka - 1216</t>
         </is>
       </c>
+      <c r="AI131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17644,6 +17859,7 @@
           <t>255/b 3rd colony, Lalkuthi, Mirpur, Mazar Road, Dhaka 1216</t>
         </is>
       </c>
+      <c r="AI132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -17795,6 +18011,7 @@
 Johar sahara bazar Road</t>
         </is>
       </c>
+      <c r="AI133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -17941,6 +18158,7 @@
           <t>68/1. Water works Road, posta, lalbagh, Dhaka - 1211</t>
         </is>
       </c>
+      <c r="AI134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -18089,6 +18307,7 @@
           <t xml:space="preserve">Abedin Villla, GA 27/4, Shahajadpur, Gulshan, Dhaka - 1212 </t>
         </is>
       </c>
+      <c r="AI135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18231,6 +18450,7 @@
           <t>83/1 Buddhijibi Road, Dhaka 1207</t>
         </is>
       </c>
+      <c r="AI136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -18376,6 +18596,7 @@
 West dhanmondi river view model town, Hajaribagh, Dhaka. </t>
         </is>
       </c>
+      <c r="AI137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -18520,6 +18741,7 @@
           <t>Uttar Khan, Dhaka.</t>
         </is>
       </c>
+      <c r="AI138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -18668,6 +18890,7 @@
           <t>151/1 Warelessgat, Mohakhali, Dhaka - 1212</t>
         </is>
       </c>
+      <c r="AI139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -18754,6 +18977,7 @@
       <c r="AF140" t="inlineStr"/>
       <c r="AG140" t="inlineStr"/>
       <c r="AH140" t="inlineStr"/>
+      <c r="AI140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18913,6 +19137,7 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18995,6 +19220,7 @@
       <c r="AF142" t="inlineStr"/>
       <c r="AG142" t="inlineStr"/>
       <c r="AH142" t="inlineStr"/>
+      <c r="AI142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -19077,6 +19303,7 @@
       <c r="AF143" t="inlineStr"/>
       <c r="AG143" t="inlineStr"/>
       <c r="AH143" t="inlineStr"/>
+      <c r="AI143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -19217,6 +19444,7 @@
           <t>36/4-A, Saheed Harez Road, Jagannathpur, Vatara, Khilkhet, Dhaka-1229.</t>
         </is>
       </c>
+      <c r="AI144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -19351,6 +19579,9 @@
           <t>295 Maxel Zaman Apartment, Dhanmondi 15, Dhaka</t>
         </is>
       </c>
+      <c r="AI145" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -19489,6 +19720,9 @@
           <t>Basic Zam Zam Tower, 171 Central Bashabo, Dhaka 1214</t>
         </is>
       </c>
+      <c r="AI146" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -19629,6 +19863,7 @@
           <t>Flat#11A, Zigatola Zenith, Zigatola, Dhaka</t>
         </is>
       </c>
+      <c r="AI147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -19769,6 +20004,7 @@
           <t>H-113, Rd-4, Mohammadi Housing Society, Adabor, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -19909,6 +20145,7 @@
           <t>House 30, Road 7, Block F, Banani, Dhaka-1213</t>
         </is>
       </c>
+      <c r="AI149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -20059,6 +20296,9 @@
           <t>308/2, Family Palacee, 3rd Floor, Shenpara, Porbota, Mitpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI150" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -20207,6 +20447,7 @@
           <t>House-Green House, Baigartek, Namapara, Shagufta, Pallabi, Dhaka</t>
         </is>
       </c>
+      <c r="AI151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -20353,6 +20594,7 @@
           <t>1769, East Jurain, Road No-1, Kadamtali, Dhaka</t>
         </is>
       </c>
+      <c r="AI152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -20493,6 +20735,7 @@
           <t>Holding#3/D/1, Flat#406, South Kallyanpur, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -20633,6 +20876,7 @@
           <t>Apt-2A, H-269, R-4/A, B-F, Bashundhara R/A, Dhaka-1229</t>
         </is>
       </c>
+      <c r="AI154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -20771,6 +21015,9 @@
           <t xml:space="preserve">house: 55 , Flat : W4  , muktijoddha sarani, East Mollertek , dakkhin khan , Uttara , Dhaka </t>
         </is>
       </c>
+      <c r="AI155" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -20911,6 +21158,7 @@
           <t xml:space="preserve">55,Proval Housing(3rd Floor North), Ring Road,Mohammadpur, Dhaka 1207. </t>
         </is>
       </c>
+      <c r="AI156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -21057,6 +21305,9 @@
           <t>House-435, Road-7, Block-C, Bashundhara R/A, Dhaka</t>
         </is>
       </c>
+      <c r="AI157" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -21193,6 +21444,7 @@
           <t>Flat- 2A, 14/3, Singapore Road, East Madartek, Dhaka-1214</t>
         </is>
       </c>
+      <c r="AI158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -21333,6 +21585,7 @@
           <t>Nahar Villa (L-4), House #32, Road#03, Mohanagar Project, W. Rampura, Dhaka</t>
         </is>
       </c>
+      <c r="AI159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -21469,6 +21722,7 @@
           <t>GP GA 169, 3rd Floor, Mohakhali School Road, Wireless Gate, Dhaka-1212.</t>
         </is>
       </c>
+      <c r="AI160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -21603,6 +21857,9 @@
           <t>House # 36, Road # 03, Block # C, Section # 12, Pallabi, Mirpur, Dhaka # 1216</t>
         </is>
       </c>
+      <c r="AI161" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -21743,6 +22000,7 @@
           <t>House # D-186 (3th floor, East), Road # 7, Mohanagar Housing Project, West Rampura, Dhaka 1219</t>
         </is>
       </c>
+      <c r="AI162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -21879,6 +22137,7 @@
           <t>Red Crescent Borak Tower -2, Level-7, 37/3/A, Eskaton Garden, Dhaka</t>
         </is>
       </c>
+      <c r="AI163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -22011,6 +22270,7 @@
           <t>House#4, Road#21, Gulshan - 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -22097,6 +22357,9 @@
       <c r="AF165" t="inlineStr"/>
       <c r="AG165" t="inlineStr"/>
       <c r="AH165" t="inlineStr"/>
+      <c r="AI165" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -22230,6 +22493,9 @@
           <t>House-3, Road-3, Block-D, Dolipara, Turag, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI166" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -22364,6 +22630,9 @@
           <t>Chocklokman, Kolony, Bogra Sadar-5800</t>
         </is>
       </c>
+      <c r="AI167" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -22498,6 +22767,9 @@
           <t>Faria &amp; Tanvir Villa, 3rd floor, Khander, Bogra-5800</t>
         </is>
       </c>
+      <c r="AI168" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -22634,6 +22906,7 @@
           <t>H N - 253 (Floor 6), West Agargaon, Dhaka</t>
         </is>
       </c>
+      <c r="AI169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -22768,6 +23041,9 @@
           <t>khander,Suttrapur road,Bogura-5800.</t>
         </is>
       </c>
+      <c r="AI170" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -22904,6 +23180,7 @@
           <t>Thonthonia,bankpara,Nazruler Basa, 2nd Floor. Bogura</t>
         </is>
       </c>
+      <c r="AI171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -23040,6 +23317,7 @@
           <t>Saujgari ,Bogra</t>
         </is>
       </c>
+      <c r="AI172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -23176,6 +23454,7 @@
           <t>Room No:101 R.B Hostel, Fuldighee, Colony, Bogra-5800</t>
         </is>
       </c>
+      <c r="AI173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -23324,6 +23603,7 @@
           <t>Village-Koyashobla, PO-Jaforpur, PS-Akkelpur, District-Joypurhat</t>
         </is>
       </c>
+      <c r="AI174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -23476,6 +23756,7 @@
           <t>Vill-Chetnapara, PO-Bhendabari, PS-Pirgonj, Rangpur</t>
         </is>
       </c>
+      <c r="AI175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -23628,6 +23909,7 @@
 Dist-Natore</t>
         </is>
       </c>
+      <c r="AI176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -23768,6 +24050,7 @@
           <t>Nataipara, Bow Bazar, Bogra Shodor-2, Ward no-21, Bogura</t>
         </is>
       </c>
+      <c r="AI177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -23902,6 +24185,9 @@
           <t>Flat # 3/702, 152/2/G-2, Eastern Pantha Chayya, Panthapath, Dhaka</t>
         </is>
       </c>
+      <c r="AI178" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -24036,6 +24322,9 @@
           <t>345/1, C-1, Ahammed Nagar, Paikpara, Mirpur-1, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI179" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -24178,6 +24467,7 @@
 Nobodoy Housing, Mohammadpur"</t>
         </is>
       </c>
+      <c r="AI180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -24318,6 +24608,7 @@
           <t>20/3(2), Dilu Road,Moghbazar,Dhaka</t>
         </is>
       </c>
+      <c r="AI181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -24468,6 +24759,9 @@
           <t>19/C, Monipuripara, Gate No-03, PS-Tejgaon, Dhaka</t>
         </is>
       </c>
+      <c r="AI182" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -24604,6 +24898,7 @@
           <t>43, Mirpur Road, Dhanmondi, Dhaka - 1205.</t>
         </is>
       </c>
+      <c r="AI183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -24740,6 +25035,7 @@
           <t>183/1/2 Moonstone properties (Flat#c-1), Green Road, Dhanmondi, Dhaka-1205.</t>
         </is>
       </c>
+      <c r="AI184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -24876,6 +25172,7 @@
           <t>Ga-103, Middle Badda. Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -25016,6 +25313,7 @@
           <t>1/D Mannu Vila, Adabor-1, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -25162,6 +25460,7 @@
           <t>GHA-1803, Mohakhali, Dhaka</t>
         </is>
       </c>
+      <c r="AI187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -25322,6 +25621,9 @@
 Uttara-10, Dhaka</t>
         </is>
       </c>
+      <c r="AI188" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -25468,6 +25770,7 @@
           <t>285/1, East Kazipara, 6th Floor, Mirpur-10, Dhaka</t>
         </is>
       </c>
+      <c r="AI189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -25602,6 +25905,9 @@
           <t>Holding-Akhaliapara,Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI190" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -25732,6 +26038,9 @@
           <t>Vill-Poshim Dorkapon,Moulvibazar Sador-3200</t>
         </is>
       </c>
+      <c r="AI191" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -25866,6 +26175,9 @@
           <t>Vill-Kayosto Gram,P.O/P.S-Fenchugonj,Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI192" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -25990,6 +26302,7 @@
         </is>
       </c>
       <c r="AH193" t="inlineStr"/>
+      <c r="AI193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -26120,6 +26433,9 @@
           <t>House#8, Road#20, Mirpur -11</t>
         </is>
       </c>
+      <c r="AI194" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -26252,6 +26568,9 @@
           <t>Zindabazar,Sylhet</t>
         </is>
       </c>
+      <c r="AI195" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -26382,6 +26701,9 @@
           <t>28/ke, Purba Noyatola, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI196" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -26514,6 +26836,7 @@
           <t>28/ke, Purba Noyatola, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -26646,6 +26969,9 @@
         </is>
       </c>
       <c r="AH198" t="inlineStr"/>
+      <c r="AI198" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -26782,6 +27108,7 @@
           <t>Vill:- Charmarddan, P.O:- Rasunia, Thana:- Sirajdikhan, Zilla:- Munshigonj</t>
         </is>
       </c>
+      <c r="AI199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -26912,6 +27239,9 @@
           <t>Vill-Boroikandi,Sylhet</t>
         </is>
       </c>
+      <c r="AI200" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -27052,6 +27382,7 @@
           <t>Jha-63,Abdul Monnaf Sarani,Middle Badda,Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -27184,6 +27515,9 @@
           <t>Vill-Bagmara,P.O/P.S-Fenchugonj,Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI202" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -27314,6 +27648,9 @@
           <t>28/ke, Purba Noyatola, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI203" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -27446,6 +27783,9 @@
           <t>28/ke, Purba Noyatola, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI204" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -27576,6 +27916,7 @@
           <t>Matarbari Project, Coxs Bazar</t>
         </is>
       </c>
+      <c r="AI205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -27670,6 +28011,9 @@
           <t>Vill-Amboekhana,Jalalabad,Sylhet</t>
         </is>
       </c>
+      <c r="AI206" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -27794,6 +28138,7 @@
 Gaibandha </t>
         </is>
       </c>
+      <c r="AI207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -27886,6 +28231,7 @@
       <c r="AF208" t="inlineStr"/>
       <c r="AG208" t="inlineStr"/>
       <c r="AH208" t="inlineStr"/>
+      <c r="AI208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -27978,6 +28324,7 @@
       <c r="AF209" t="inlineStr"/>
       <c r="AG209" t="inlineStr"/>
       <c r="AH209" t="inlineStr"/>
+      <c r="AI209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -28100,6 +28447,7 @@
           <t>Ward-8, Boiddogona, Coxs Bazar Sadar, Coxs Bazar</t>
         </is>
       </c>
+      <c r="AI210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -28222,6 +28570,7 @@
           <t xml:space="preserve">Village- Noya Tilla, PO/PS- Fenchugonj, Sylhet </t>
         </is>
       </c>
+      <c r="AI211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -28342,6 +28691,7 @@
           <t>Alubdi, Choto Masjid Road, Eastern housing, Pallabi 2nd phase, Mirpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -28460,6 +28810,7 @@
           <t>2nd Floor, Shuhel Village, Nobab Road, Sylhet</t>
         </is>
       </c>
+      <c r="AI213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -28596,6 +28947,7 @@
           <t>Chayatoru-30, Rahman Villa , Lamabazar, Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -28736,6 +29088,7 @@
           <t>Ruman Villa ; House # 1 ; Road # 4 ; Shamimabad R/A ; Kanishail Rd. South Bagbari ; Sylhet</t>
         </is>
       </c>
+      <c r="AI215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -28872,6 +29225,7 @@
           <t>House # 2 ; Road # 3 ; Block - C ; Shapla Bag ; Tilagor ; Sylhet</t>
         </is>
       </c>
+      <c r="AI216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -29006,6 +29360,9 @@
           <t>Radient Darul Abrar, Flat # 4B, House # 634, Road # 5/1, Block-B, Banasree, Dhaka-1219</t>
         </is>
       </c>
+      <c r="AI217" t="n">
+        <v>263</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -29139,6 +29496,9 @@
         <is>
           <t>161/7, Baganbari, North Bashantek, Dhaka Cantonment,  Dhaka-1206</t>
         </is>
+      </c>
+      <c r="AI218" t="n">
+        <v>263</v>
       </c>
     </row>
     <row r="219">
@@ -29228,6 +29588,7 @@
       <c r="AF219" t="inlineStr"/>
       <c r="AG219" t="inlineStr"/>
       <c r="AH219" t="inlineStr"/>
+      <c r="AI219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -29316,6 +29677,7 @@
       <c r="AF220" t="inlineStr"/>
       <c r="AG220" t="inlineStr"/>
       <c r="AH220" t="inlineStr"/>
+      <c r="AI220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -29468,6 +29830,9 @@
           <t>Alvi Villa (4th Floor), KA-112/7, South Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI221" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -29614,6 +29979,7 @@
           <t>House-324/2, Floor-7/A, Sornolota, Kawla, Dokkinkhan, Jamtola, Dhaka</t>
         </is>
       </c>
+      <c r="AI222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -29744,6 +30110,9 @@
           <t>Red Crescent Borak Tower -2, Level-7, 37/3/A, Eskaton Garden, Dhaka</t>
         </is>
       </c>
+      <c r="AI223" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -29878,6 +30247,7 @@
           <t>Vill-Jaingail,P.O-Tukerbazar,P.S-Jalalabad,Distric-Sylhet</t>
         </is>
       </c>
+      <c r="AI224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -30012,6 +30382,9 @@
           <t>332/1,Shewrapar.Mirpur.Dhaka</t>
         </is>
       </c>
+      <c r="AI225" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -30146,6 +30519,7 @@
           <t>Vill-Daudpur,P.O-Ranga Daudpur,P.S-Muglabazar,Distric-Sylhet</t>
         </is>
       </c>
+      <c r="AI226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -30272,6 +30646,9 @@
           <t>Red Crescent Borak Tower -2, Level-7, 37/3/A, Eskaton Garden, Dhaka</t>
         </is>
       </c>
+      <c r="AI227" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -30402,6 +30779,9 @@
           <t>10/C, Malibagh Chowdhurypara, Dhaka</t>
         </is>
       </c>
+      <c r="AI228" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -30534,6 +30914,7 @@
           <t>Hatirjheel Modhubag,</t>
         </is>
       </c>
+      <c r="AI229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -30666,6 +31047,9 @@
           <t>Akupara, Ashulia, Savar, Dhaka</t>
         </is>
       </c>
+      <c r="AI230" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -30794,6 +31178,7 @@
           <t>Dhaka</t>
         </is>
       </c>
+      <c r="AI231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -30880,6 +31265,9 @@
       <c r="AF232" t="inlineStr"/>
       <c r="AG232" t="inlineStr"/>
       <c r="AH232" t="inlineStr"/>
+      <c r="AI232" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -31034,6 +31422,7 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -31188,6 +31577,7 @@
 Jamalpur</t>
         </is>
       </c>
+      <c r="AI234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -31319,6 +31709,7 @@
           <t>6/1, West Agargaon, Sher-e-Bangla Nagar, Dhaka</t>
         </is>
       </c>
+      <c r="AI235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -31459,6 +31850,7 @@
           <t>Jamai Bazar, Korail, Banani, Dhaka</t>
         </is>
       </c>
+      <c r="AI236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -31585,6 +31977,7 @@
           <t>Village-Gerakhali, PO-Islamabad, Dist-Patuakhali</t>
         </is>
       </c>
+      <c r="AI237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -31707,6 +32100,7 @@
           <t>House-10, Road-2, Adabor, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -31791,6 +32185,7 @@
       <c r="AF239" t="inlineStr"/>
       <c r="AG239" t="inlineStr"/>
       <c r="AH239" t="inlineStr"/>
+      <c r="AI239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -31921,6 +32316,9 @@
           <t>Atim School Road, 14/3 Bagbari Sylhet-3100.</t>
         </is>
       </c>
+      <c r="AI240" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -32055,6 +32453,9 @@
           <t>Mannan House ; 84/A Waves ; Amberkhana ; Sylhet</t>
         </is>
       </c>
+      <c r="AI241" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -32189,6 +32590,9 @@
           <t>Bondhon13/C,Block-C,Akhalia,Nuapara,Sylhet</t>
         </is>
       </c>
+      <c r="AI242" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -32322,6 +32726,9 @@
         <is>
           <t>Vill-Gobindosri,House no-8,Kusumbag,Moulvibazar-3200</t>
         </is>
+      </c>
+      <c r="AI243" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="244">
@@ -32447,6 +32854,9 @@
           <t>12 Kajol Shah, Block # B, Medecal Road, Sylhet</t>
         </is>
       </c>
+      <c r="AI244" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -32581,6 +32991,9 @@
           <t>KA-197/2, Uttarpar,Khilkhet, Dhaka</t>
         </is>
       </c>
+      <c r="AI245" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -32715,6 +33128,9 @@
           <t>1/1 H, Mirbagh, Noyatola, Mogbazar, Ramna, Dhaka</t>
         </is>
       </c>
+      <c r="AI246" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -32852,6 +33268,9 @@
 "</t>
         </is>
       </c>
+      <c r="AI247" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -32990,6 +33409,9 @@
           <t>Flat#6B, House#60, Road#03, Block#D, Mohanagor Project, Rampura, Dhaka.</t>
         </is>
       </c>
+      <c r="AI248" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -33124,6 +33546,9 @@
           <t>330/k ,East Nakhal Para, Tejgaon.</t>
         </is>
       </c>
+      <c r="AI249" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -33258,6 +33683,9 @@
           <t>1/1, H, 4th Floor, Mirbaug, Noyatola, Dhaka-1217</t>
         </is>
       </c>
+      <c r="AI250" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -33392,6 +33820,9 @@
           <t>JA-63,Abdul Monnaf Sarani,Middle Badda,Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI251" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -33525,6 +33956,9 @@
         <is>
           <t>Shapnakothir, Taraboniarachara, Kabarstan Road, Cox's Bazar</t>
         </is>
+      </c>
+      <c r="AI252" t="n">
+        <v>207</v>
       </c>
     </row>
     <row r="253">
@@ -33612,6 +34046,9 @@
       <c r="AF253" t="inlineStr"/>
       <c r="AG253" t="inlineStr"/>
       <c r="AH253" t="inlineStr"/>
+      <c r="AI253" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -33698,6 +34135,9 @@
       <c r="AF254" t="inlineStr"/>
       <c r="AG254" t="inlineStr"/>
       <c r="AH254" t="inlineStr"/>
+      <c r="AI254" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -33846,6 +34286,7 @@
           <t>House-2, road-3, Akota R/A, Satarkul Road, North Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -33990,6 +34431,7 @@
           <t>Bekinagor, Daudkandi, Gram Raipur-3519, Cumilla</t>
         </is>
       </c>
+      <c r="AI256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -34128,6 +34570,7 @@
 Patuakhali</t>
         </is>
       </c>
+      <c r="AI257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -34264,6 +34707,7 @@
 Rajbari</t>
         </is>
       </c>
+      <c r="AI258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -34412,6 +34856,7 @@
           <t>59/1, Durga Mandir Goli, Jafrabad, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -34558,6 +35003,7 @@
           <t>Block-F, Road-10, House-175, Bashundhara R/A, Dhaka</t>
         </is>
       </c>
+      <c r="AI260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -34713,6 +35159,7 @@
           <t>215/4/A/3, East Rampura, Dhaka</t>
         </is>
       </c>
+      <c r="AI261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -34857,6 +35304,7 @@
           <t>Mogbazar, Hatirjheel, Dhaka</t>
         </is>
       </c>
+      <c r="AI262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -35008,6 +35456,7 @@
 Kurigram</t>
         </is>
       </c>
+      <c r="AI263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -35156,6 +35605,9 @@
           <t>Road-2, House-17, Sector-7, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI264" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -35304,6 +35756,7 @@
           <t>House-7, Road-2, Lalkuthi Bazar, First Colony, Mirpur-1, Dhaka</t>
         </is>
       </c>
+      <c r="AI265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -35450,6 +35903,7 @@
           <t>Janata Housing, H-121, R-7, Mirpur-2, Dhaka</t>
         </is>
       </c>
+      <c r="AI266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -35542,6 +35996,7 @@
       <c r="AF267" t="inlineStr"/>
       <c r="AG267" t="inlineStr"/>
       <c r="AH267" t="inlineStr"/>
+      <c r="AI267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -35674,6 +36129,7 @@
 Dist-Kustia</t>
         </is>
       </c>
+      <c r="AI268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -35810,6 +36266,7 @@
           <t>House# 294/1, Road# 8/A, Dhanmondi,Dhaka</t>
         </is>
       </c>
+      <c r="AI269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -35950,6 +36407,7 @@
           <t>6/A, Shantikunjo R/A, New Eskaton,Dhaka</t>
         </is>
       </c>
+      <c r="AI270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -36088,6 +36546,9 @@
           <t>Gulshan-badda link road</t>
         </is>
       </c>
+      <c r="AI271" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -36224,6 +36685,7 @@
           <t>Road- 25/A, House- 91, Banani, Dhaka</t>
         </is>
       </c>
+      <c r="AI272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -36358,6 +36820,9 @@
           <t>House # 6, Road # 3/1, Al Madina R/A, Shahporan, Sylhet</t>
         </is>
       </c>
+      <c r="AI273" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -36506,6 +36971,7 @@
           <t>House#21,Road#04,Sector#04,Uttara,Dhaka-1230</t>
         </is>
       </c>
+      <c r="AI274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -36642,6 +37108,7 @@
           <t>C/O- Md. Ashraf Ali, House No: 06, Lane: 01, Road: Masjid road 04, Satarkul West Padardia. P.O: Gulshan, P.S: Badda, Dhaka-1212.</t>
         </is>
       </c>
+      <c r="AI275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -36774,6 +37241,7 @@
           <t>Ground Floor,Builiding No- G-24/1, Fokirapul T&amp;T Colony, Dhaka</t>
         </is>
       </c>
+      <c r="AI276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -36914,6 +37382,7 @@
           <t xml:space="preserve">House no. 01, Road no. 05, Adarshabag, Farmer More, Jatrabari, Dhaka-1362.  </t>
         </is>
       </c>
+      <c r="AI277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -37050,6 +37519,7 @@
           <t>House-11;Road-11,North Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -37179,6 +37649,9 @@
         <is>
           <t>28/ke, Purba Noyatola, Moghbazar, Dhaka</t>
         </is>
+      </c>
+      <c r="AI279" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="280">
@@ -37268,6 +37741,7 @@
       <c r="AF280" t="inlineStr"/>
       <c r="AG280" t="inlineStr"/>
       <c r="AH280" t="inlineStr"/>
+      <c r="AI280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -37406,6 +37880,7 @@
           <t>Village- Amo Tea Estate, PO- Chandpur, Dist- Hobigonj</t>
         </is>
       </c>
+      <c r="AI281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -37556,6 +38031,7 @@
           <t>10/A, Eastern Corner, Circuit House Road, Shantinagar, Dhaka</t>
         </is>
       </c>
+      <c r="AI282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -37709,6 +38185,7 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -37861,6 +38338,7 @@
 Dist-Noakhali</t>
         </is>
       </c>
+      <c r="AI284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -38009,6 +38487,7 @@
           <t>Road-3, House-32, Nikunja-2, Khilkhet, Dhaka</t>
         </is>
       </c>
+      <c r="AI285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -38159,6 +38638,9 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI286" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -38306,6 +38788,7 @@
 Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -38458,6 +38941,9 @@
           <t>House-8, Road-7/A, Tanjim Building, Sejanadarbagh, Adorshonogor, Middle Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI288" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -38602,6 +39088,7 @@
           <t>House- JA-108/1, Moddha badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -38720,6 +39207,7 @@
       <c r="AF290" t="inlineStr"/>
       <c r="AG290" t="inlineStr"/>
       <c r="AH290" t="inlineStr"/>
+      <c r="AI290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -38862,6 +39350,7 @@
           <t>House-61, Road-3, Sector-13, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -39008,6 +39497,7 @@
           <t>House-123/3, Matabbar Road, North Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -39156,6 +39646,7 @@
           <t>177/2 Boubazar, Gulshan 1, Dhaka</t>
         </is>
       </c>
+      <c r="AI293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -39302,6 +39793,7 @@
           <t>House-KA-115/20, South Mohakhali, Dhaka</t>
         </is>
       </c>
+      <c r="AI294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -39420,6 +39912,7 @@
           <t>Gobindapur, Habiganj</t>
         </is>
       </c>
+      <c r="AI295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -39546,6 +40039,7 @@
           <t>Village-Gerakhali, PO-Islamabad, Patuakhali Sadar, Patuakhali</t>
         </is>
       </c>
+      <c r="AI296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -39694,6 +40188,7 @@
           <t>1383/10, Natunbag, Khilgaon, dhaka</t>
         </is>
       </c>
+      <c r="AI297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -39842,6 +40337,7 @@
           <t xml:space="preserve">67, West Nakhal Para, Tejgaon, Dhaka </t>
         </is>
       </c>
+      <c r="AI298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -39988,6 +40484,7 @@
           <t>249/A, East Nakhalpara, Tejgaon, Dhaka</t>
         </is>
       </c>
+      <c r="AI299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -40134,6 +40631,7 @@
           <t>House-Dolapara, Village-Dorgapara, PO-Parbotipur-5250, Dist-Dinajpur</t>
         </is>
       </c>
+      <c r="AI300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -40264,6 +40762,7 @@
           <t>House-189, Mollartek, Dakhin Khan, Uttara, Dhaka</t>
         </is>
       </c>
+      <c r="AI301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -40400,6 +40899,7 @@
           <t>Road-7,  House-5, Block-G, Arifabad Housing, Dhaka-1215</t>
         </is>
       </c>
+      <c r="AI302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -40540,6 +41040,7 @@
           <t>Adarshabag, Konapara, Jatrabari, Dhaka</t>
         </is>
       </c>
+      <c r="AI303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -40676,6 +41177,7 @@
           <t>45/13, Jalalabad R/A, Sylhet</t>
         </is>
       </c>
+      <c r="AI304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -40812,6 +41314,7 @@
           <t>1st Floor 2B, Zihan House, 428/C/2, Garden View Road, South Paik Para, Mirpur, Dhaka.</t>
         </is>
       </c>
+      <c r="AI305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -40952,6 +41455,7 @@
           <t>509/Cha, Chamiman Goli, Noyatola, Ambagan, Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -41088,6 +41592,7 @@
           <t>107-Razargoly, Dorgamoholla, Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -41222,6 +41727,9 @@
           <t>House: 29/4, Block : A Kumar Para, Sylhet-3100</t>
         </is>
       </c>
+      <c r="AI308" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -41358,6 +41866,7 @@
           <t>Village : Sabuj Bug (behind Agriculture Farm); Bogura Sadar; Bogura</t>
         </is>
       </c>
+      <c r="AI309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -41490,6 +41999,7 @@
           <t>Faridpur, P.O: Amdabad Bazar, P.S: Kotwali, Jashore</t>
         </is>
       </c>
+      <c r="AI310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -41630,6 +42140,7 @@
           <t>27/1 West Dolairpar, Ali Hossain road Shaympur, Dhaka 1204</t>
         </is>
       </c>
+      <c r="AI311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -41766,6 +42277,7 @@
           <t>181/2,Noyatola,Moghbazar,Dhaka</t>
         </is>
       </c>
+      <c r="AI312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -41856,6 +42368,9 @@
       <c r="AF313" t="inlineStr"/>
       <c r="AG313" t="inlineStr"/>
       <c r="AH313" t="inlineStr"/>
+      <c r="AI313" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -41948,6 +42463,7 @@
       <c r="AF314" t="inlineStr"/>
       <c r="AG314" t="inlineStr"/>
       <c r="AH314" t="inlineStr"/>
+      <c r="AI314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -42036,6 +42552,7 @@
       <c r="AF315" t="inlineStr"/>
       <c r="AG315" t="inlineStr"/>
       <c r="AH315" t="inlineStr"/>
+      <c r="AI315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -42176,6 +42693,7 @@
       </c>
       <c r="AG316" t="inlineStr"/>
       <c r="AH316" t="inlineStr"/>
+      <c r="AI316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -42268,6 +42786,7 @@
       <c r="AF317" t="inlineStr"/>
       <c r="AG317" t="inlineStr"/>
       <c r="AH317" t="inlineStr"/>
+      <c r="AI317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -42354,6 +42873,9 @@
       <c r="AF318" t="inlineStr"/>
       <c r="AG318" t="inlineStr"/>
       <c r="AH318" t="inlineStr"/>
+      <c r="AI318" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -42442,6 +42964,7 @@
       <c r="AF319" t="inlineStr"/>
       <c r="AG319" t="inlineStr"/>
       <c r="AH319" t="inlineStr"/>
+      <c r="AI319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -42588,6 +43111,7 @@
           <t>Flat-4/3, House-30/F, Road-4, Cantonment, Dhaka</t>
         </is>
       </c>
+      <c r="AI320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -42734,6 +43258,7 @@
           <t>Road-1, Block-B, House-3, Nobodoy Housing, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -42872,6 +43397,7 @@
           <t>517, Pardogair, Natunpara (DND Road), Demra, Dhaka</t>
         </is>
       </c>
+      <c r="AI322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -43020,6 +43546,7 @@
           <t>545, North Kafrul, Dhaka</t>
         </is>
       </c>
+      <c r="AI323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -43146,6 +43673,7 @@
           <t>Village-Latifpur, PO-Sylhet Sadar, South Surma, Sylhet</t>
         </is>
       </c>
+      <c r="AI324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -43298,6 +43826,7 @@
           <t>Baitul Ahabab, House-424, Bagun Bari, Shadhinata sharani Link Road, Badda, dhaka</t>
         </is>
       </c>
+      <c r="AI325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -43448,6 +43977,7 @@
 </t>
         </is>
       </c>
+      <c r="AI326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -43598,6 +44128,9 @@
 TB Gate, Mohakhali, Dhaka</t>
         </is>
       </c>
+      <c r="AI327" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -43727,6 +44260,9 @@
         <is>
           <t>House#4, Road#21, Gulshan 1- Dhaka</t>
         </is>
+      </c>
+      <c r="AI328" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="329">
@@ -43814,6 +44350,9 @@
       <c r="AF329" t="inlineStr"/>
       <c r="AG329" t="inlineStr"/>
       <c r="AH329" t="inlineStr"/>
+      <c r="AI329" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -43900,6 +44439,9 @@
       <c r="AF330" t="inlineStr"/>
       <c r="AG330" t="inlineStr"/>
       <c r="AH330" t="inlineStr"/>
+      <c r="AI330" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -43988,6 +44530,7 @@
       <c r="AF331" t="inlineStr"/>
       <c r="AG331" t="inlineStr"/>
       <c r="AH331" t="inlineStr"/>
+      <c r="AI331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -44133,6 +44676,9 @@
           <t>333, Nayanagar Uttar, Gulshan, Dhaka</t>
         </is>
       </c>
+      <c r="AI332" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -44287,6 +44833,9 @@
 154/5, 1st Floor, Shonkor, Mohammadpur, Dhaka </t>
         </is>
       </c>
+      <c r="AI333" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -44437,6 +44986,7 @@
           <t>Nilganj Shah Para, Holding No-701, Jessore Sadar, Jessore</t>
         </is>
       </c>
+      <c r="AI334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -44583,6 +45133,9 @@
           <t>Aukhpara, Ashulia, Savar, Dhaka</t>
         </is>
       </c>
+      <c r="AI335" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -44717,6 +45270,9 @@
           <t>15/2, 4th floor,  Ali &amp; Noor Real State, Mohammadpur, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI336" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -44847,6 +45403,9 @@
           <t>276D, Boro Moghbazar, Dhaka</t>
         </is>
       </c>
+      <c r="AI337" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -44977,6 +45536,9 @@
           <t>Maniknogor, Dhaka</t>
         </is>
       </c>
+      <c r="AI338" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -45113,6 +45675,7 @@
           <t>Badda, Gulshan, Dhaka</t>
         </is>
       </c>
+      <c r="AI339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -45247,6 +45810,9 @@
           <t>Holding no-54/A, Soto boyra puja khola, GPO 9000, Sonadanga Khulna</t>
         </is>
       </c>
+      <c r="AI340" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -45383,6 +45949,7 @@
           <t>Moghbazar, Modhubagh</t>
         </is>
       </c>
+      <c r="AI341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -45517,6 +46084,9 @@
           <t>Moroli (infront of jora mondir), Kotwali, Jashore</t>
         </is>
       </c>
+      <c r="AI342" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -45657,6 +46227,7 @@
           <t>Flat#F8, House#19, Road#7, Block#F, Banasree, Rampura, Dhaka-1219</t>
         </is>
       </c>
+      <c r="AI343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -45787,6 +46358,9 @@
           <t>Badda, Gulshan, Dhaka</t>
         </is>
       </c>
+      <c r="AI344" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -45921,6 +46495,9 @@
           <t>Dakatia, Nouda, Jessore</t>
         </is>
       </c>
+      <c r="AI345" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -46051,6 +46628,9 @@
           <t>Malibagh, Dhaka</t>
         </is>
       </c>
+      <c r="AI346" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -46181,6 +46761,9 @@
           <t>Rampura, Banasree, E Block</t>
         </is>
       </c>
+      <c r="AI347" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -46317,6 +46900,7 @@
           <t>Basila,West Dhanmondi, Road No 9,Block-B,House no-19</t>
         </is>
       </c>
+      <c r="AI348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -46449,6 +47033,7 @@
           <t>Badda, Gulshan, Dhaka</t>
         </is>
       </c>
+      <c r="AI349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -46578,6 +47163,9 @@
         <is>
           <t>Tongi Bazar, Tongi Gazipur</t>
         </is>
+      </c>
+      <c r="AI350" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="351">
@@ -46671,6 +47259,7 @@
       <c r="AF351" t="inlineStr"/>
       <c r="AG351" t="inlineStr"/>
       <c r="AH351" t="inlineStr"/>
+      <c r="AI351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -46801,6 +47390,9 @@
           <t>C. T. College Para, Jessore</t>
         </is>
       </c>
+      <c r="AI352" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -46939,6 +47531,9 @@
       </c>
       <c r="AG353" t="inlineStr"/>
       <c r="AH353" t="inlineStr"/>
+      <c r="AI353" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -47093,6 +47688,9 @@
 Dhaka</t>
         </is>
       </c>
+      <c r="AI354" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -47242,6 +47840,9 @@
           <t>House No- KA/41/9/C, Ferdous Villa, Kala Chandpur, Nadda, Dhaka</t>
         </is>
       </c>
+      <c r="AI355" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -47388,6 +47989,9 @@
           <t>Vill/PO-Tulshighat, PS-Sadar, Dist-Gaibandha</t>
         </is>
       </c>
+      <c r="AI356" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -47536,6 +48140,7 @@
           <t>House-59, Road-3, Block-A, Aftabnagar, Dhaka</t>
         </is>
       </c>
+      <c r="AI357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -47686,6 +48291,9 @@
           <t>Vill: Bordha, PO: Choriar bil bazar, PS: Soilokupa, Jhenidah</t>
         </is>
       </c>
+      <c r="AI358" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -47836,6 +48444,9 @@
           <t>Saitalia, Tengra, Sreepur, Gazipur</t>
         </is>
       </c>
+      <c r="AI359" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -47986,6 +48597,9 @@
           <t>H-16/5, Modhubag, Ward-6, Ramna, Dhaka</t>
         </is>
       </c>
+      <c r="AI360" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -48132,6 +48746,9 @@
           <t>135/18, West Nandipara, Modina Shorok, South Banasree, Titash Stand, Leguna Stand, Dhaka</t>
         </is>
       </c>
+      <c r="AI361" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -48278,6 +48895,9 @@
           <t>House-17, Block-C, Road-2, Banasree, Rampura, Dhaka</t>
         </is>
       </c>
+      <c r="AI362" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -48430,6 +49050,9 @@
           <t>House-184, Ekrampur, Shomvopara, Sonargaon, Narayangonj</t>
         </is>
       </c>
+      <c r="AI363" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -48576,6 +49199,9 @@
           <t>63/3, Brahmanchiron, Dholpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI364" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -48722,6 +49348,9 @@
           <t>House-171 (Ahsan Heritage), Road- Bin Protik, Sayed Nagor, Vatara, Dhaka-1212</t>
         </is>
       </c>
+      <c r="AI365" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -48864,6 +49493,9 @@
           <t>Sumon Villa, Arju Goli, Adorsho Nogor, Uttor Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI366" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -49006,6 +49638,9 @@
           <t>House-7, Road-2, Chad Uddan, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI367" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -49144,6 +49779,9 @@
           <t>TA-79, Amble Rowshan, Middle Badda, Dhaka</t>
         </is>
       </c>
+      <c r="AI368" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -49278,6 +49916,9 @@
           <t>House-4, Road-9/1, Block-E, Section-12, Mirpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI369" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -49412,6 +50053,9 @@
           <t>18, Darussalam, Mirpur, Dhaka-1216</t>
         </is>
       </c>
+      <c r="AI370" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -49560,6 +50204,7 @@
           <t>13, Katasur, Sher-E-Bangla Road, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -49708,6 +50353,9 @@
 Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI372" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -49842,6 +50490,9 @@
           <t>Flat # 2A, House # 273/A, Road # 05, Mohammadi Housing Society, Mohammadpur, Dhaka-1207</t>
         </is>
       </c>
+      <c r="AI373" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -49976,6 +50627,9 @@
           <t>Village : Dogair East Para ,PO Sarulia, PS : Demra ,District : Dhaka</t>
         </is>
       </c>
+      <c r="AI374" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -50109,6 +50763,9 @@
         <is>
           <t>Arobi Vila (2nd Floor), Sarkar Bari (Near Jame Mosjid), Vatara, Dhaka-1229</t>
         </is>
+      </c>
+      <c r="AI375" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="376">
@@ -50198,6 +50855,7 @@
       <c r="AF376" t="inlineStr"/>
       <c r="AG376" t="inlineStr"/>
       <c r="AH376" t="inlineStr"/>
+      <c r="AI376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -50344,6 +51002,9 @@
           <t>111/3 A, North Mugda Pra, Dhaka</t>
         </is>
       </c>
+      <c r="AI377" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -50492,6 +51153,7 @@
           <t>1769, East Jurain, Kadomtoli, Dhaka-1204</t>
         </is>
       </c>
+      <c r="AI378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -50638,6 +51300,9 @@
           <t>PC culture society, Shekhertek, Road-9, House-48, Mohammadpur, Dhaka</t>
         </is>
       </c>
+      <c r="AI379" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -50784,6 +51449,9 @@
           <t>139/9, Middle Paikpara, Mirpur-1, Dhaka</t>
         </is>
       </c>
+      <c r="AI380" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -50920,6 +51588,7 @@
           <t>Akupara, Ashulia, Savar, Dhaka</t>
         </is>
       </c>
+      <c r="AI381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -51052,6 +51721,7 @@
           <t>House - 755 (5th Floor), Road #23, Block # G, Bashundhara R/A, Vatara, Dhaka - 1229.</t>
         </is>
       </c>
+      <c r="AI382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -51140,6 +51810,7 @@
       <c r="AF383" t="inlineStr"/>
       <c r="AG383" t="inlineStr"/>
       <c r="AH383" t="inlineStr"/>
+      <c r="AI383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -51286,6 +51957,7 @@
           <t>Flat # A7, H # 6, Level - 7, Block # H, Pallabi Extension R/A, Mirpur Dhaka - 1216.</t>
         </is>
       </c>
+      <c r="AI384" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>